<commit_message>
feat(labtest): update feature and excel utilities for data reading
</commit_message>
<xml_diff>
--- a/src/test/resources/Reader/Apollo247_TestData.xlsx
+++ b/src/test/resources/Reader/Apollo247_TestData.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shyam Sundar\OneDrive\Desktop\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F3F67F-6C32-4105-A278-178A7104CA5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="BMI" sheetId="1" r:id="rId1"/>
+    <sheet name="Patients_Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,12 +25,156 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="41">
+  <si>
+    <t>Height (ft)</t>
+  </si>
+  <si>
+    <t>Weight (kg)</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Underweight</t>
+  </si>
+  <si>
+    <t>Overweight</t>
+  </si>
+  <si>
+    <t>Obese</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>DateOfBirth</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Relation</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Brother</t>
+  </si>
+  <si>
+    <t>rahul.kumar@gmail.com</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>Sharma</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Sister</t>
+  </si>
+  <si>
+    <t>priya.sharma@gmail.com</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>Reddy</t>
+  </si>
+  <si>
+    <t>Father</t>
+  </si>
+  <si>
+    <t>arjun.reddy@gmail.com</t>
+  </si>
+  <si>
+    <t>Lakshmi</t>
+  </si>
+  <si>
+    <t>Devi</t>
+  </si>
+  <si>
+    <t>Mother</t>
+  </si>
+  <si>
+    <t>lakshmi.devi@gmail.com</t>
+  </si>
+  <si>
+    <t>Kiran</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Son</t>
+  </si>
+  <si>
+    <t>kiran.kumar@gmail.com</t>
+  </si>
+  <si>
+    <t>TestName</t>
+  </si>
+  <si>
+    <t>CBC Test</t>
+  </si>
+  <si>
+    <t>PPBS Test</t>
+  </si>
+  <si>
+    <t>FBS Test</t>
+  </si>
+  <si>
+    <t>Hemogram Test</t>
+  </si>
+  <si>
+    <t>vitamin D Test</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -37,7 +188,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,14 +196,52 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +519,299 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.08984375" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>5.7</v>
+      </c>
+      <c r="B2" s="2">
+        <v>65</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2">
+        <v>50</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="B4" s="2">
+        <v>70</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>5.8</v>
+      </c>
+      <c r="B5" s="2">
+        <v>80</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5.2</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6.1</v>
+      </c>
+      <c r="B7" s="2">
+        <v>90</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>5.9</v>
+      </c>
+      <c r="B9" s="2">
+        <v>75</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>5.7</v>
+      </c>
+      <c r="B10" s="2">
+        <v>101</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>6</v>
+      </c>
+      <c r="B11" s="2">
+        <v>106</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FECFBD-25D6-4F6C-91BB-5A6C18ADD79D}">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="5">
+        <v>36022</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="5">
+        <v>36607</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="5">
+        <v>35008</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="5">
+        <v>27406</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="5">
+        <v>40359</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G6" r:id="rId1" display="mailto:kiran.kumar@gmail.com" xr:uid="{8E4FF1C4-A486-4E00-8CAC-5B0751AA02CA}"/>
+    <hyperlink ref="G5" r:id="rId2" display="mailto:lakshmi.devi@gmail.com" xr:uid="{56886F69-2DA0-4471-BC73-857F2BD266E1}"/>
+    <hyperlink ref="G4" r:id="rId3" display="mailto:arjun.reddy@gmail.com" xr:uid="{E81D8ACA-4202-454E-88EE-0DC02BFA7560}"/>
+    <hyperlink ref="G3" r:id="rId4" display="mailto:priya.sharma@gmail.com" xr:uid="{1D8F99EF-3E43-4DDA-98DA-3BF0942722F8}"/>
+    <hyperlink ref="G2" r:id="rId5" display="mailto:rahul.kumar@gmail.com" xr:uid="{3AFE8805-37A3-476D-8A50-2E016D8D5CA8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(labtest): handled dynamic elements and improved test stability
</commit_message>
<xml_diff>
--- a/src/test/resources/Reader/Apollo247_TestData.xlsx
+++ b/src/test/resources/Reader/Apollo247_TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shyam Sundar\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F3F67F-6C32-4105-A278-178A7104CA5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F873BA-3D4E-4150-8BD9-A29E317C2ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
   <si>
     <t>Height (ft)</t>
   </si>
@@ -131,24 +131,6 @@
   </si>
   <si>
     <t>kiran.kumar@gmail.com</t>
-  </si>
-  <si>
-    <t>TestName</t>
-  </si>
-  <si>
-    <t>CBC Test</t>
-  </si>
-  <si>
-    <t>PPBS Test</t>
-  </si>
-  <si>
-    <t>FBS Test</t>
-  </si>
-  <si>
-    <t>Hemogram Test</t>
-  </si>
-  <si>
-    <t>vitamin D Test</t>
   </si>
 </sst>
 </file>
@@ -656,161 +638,142 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FECFBD-25D6-4F6C-91BB-5A6C18ADD79D}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="5">
+      <c r="C2" s="5">
         <v>36022</v>
       </c>
+      <c r="D2" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="E2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="5">
+        <v>36607</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="5">
+        <v>35008</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="5">
-        <v>36607</v>
-      </c>
-      <c r="E3" s="4" t="s">
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="5">
+        <v>27406</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="5">
-        <v>35008</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="5">
-        <v>27406</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="5">
+      <c r="C6" s="5">
         <v>40359</v>
       </c>
+      <c r="D6" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="E6" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G6" r:id="rId1" display="mailto:kiran.kumar@gmail.com" xr:uid="{8E4FF1C4-A486-4E00-8CAC-5B0751AA02CA}"/>
-    <hyperlink ref="G5" r:id="rId2" display="mailto:lakshmi.devi@gmail.com" xr:uid="{56886F69-2DA0-4471-BC73-857F2BD266E1}"/>
-    <hyperlink ref="G4" r:id="rId3" display="mailto:arjun.reddy@gmail.com" xr:uid="{E81D8ACA-4202-454E-88EE-0DC02BFA7560}"/>
-    <hyperlink ref="G3" r:id="rId4" display="mailto:priya.sharma@gmail.com" xr:uid="{1D8F99EF-3E43-4DDA-98DA-3BF0942722F8}"/>
-    <hyperlink ref="G2" r:id="rId5" display="mailto:rahul.kumar@gmail.com" xr:uid="{3AFE8805-37A3-476D-8A50-2E016D8D5CA8}"/>
+    <hyperlink ref="F6" r:id="rId1" display="mailto:kiran.kumar@gmail.com" xr:uid="{8E4FF1C4-A486-4E00-8CAC-5B0751AA02CA}"/>
+    <hyperlink ref="F5" r:id="rId2" display="mailto:lakshmi.devi@gmail.com" xr:uid="{56886F69-2DA0-4471-BC73-857F2BD266E1}"/>
+    <hyperlink ref="F4" r:id="rId3" display="mailto:arjun.reddy@gmail.com" xr:uid="{E81D8ACA-4202-454E-88EE-0DC02BFA7560}"/>
+    <hyperlink ref="F3" r:id="rId4" display="mailto:priya.sharma@gmail.com" xr:uid="{1D8F99EF-3E43-4DDA-98DA-3BF0942722F8}"/>
+    <hyperlink ref="F2" r:id="rId5" display="mailto:rahul.kumar@gmail.com" xr:uid="{3AFE8805-37A3-476D-8A50-2E016D8D5CA8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added test cart page and improved lab test booking flow with updated data and reports
</commit_message>
<xml_diff>
--- a/src/test/resources/Reader/Apollo247_TestData.xlsx
+++ b/src/test/resources/Reader/Apollo247_TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shyam Sundar\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F873BA-3D4E-4150-8BD9-A29E317C2ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE1200AA-3320-4C2B-BF0F-F0EE70AC6368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
   <si>
     <t>Height (ft)</t>
   </si>
@@ -131,13 +131,28 @@
   </si>
   <si>
     <t>kiran.kumar@gmail.com</t>
+  </si>
+  <si>
+    <t>12/03/2002</t>
+  </si>
+  <si>
+    <t>12/03/2006</t>
+  </si>
+  <si>
+    <t>15/02/2000</t>
+  </si>
+  <si>
+    <t>12/11/1998</t>
+  </si>
+  <si>
+    <t>01/07/2008</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -157,6 +172,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -212,14 +233,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -647,7 +668,7 @@
     <col min="6" max="6" width="22.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
@@ -674,8 +695,8 @@
       <c r="B2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="5">
-        <v>36022</v>
+      <c r="C2" s="7" t="s">
+        <v>35</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>15</v>
@@ -683,7 +704,7 @@
       <c r="E2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -694,8 +715,8 @@
       <c r="B3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="5">
-        <v>36607</v>
+      <c r="C3" s="7" t="s">
+        <v>37</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>20</v>
@@ -703,7 +724,7 @@
       <c r="E3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>22</v>
       </c>
     </row>
@@ -714,8 +735,8 @@
       <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="5">
-        <v>35008</v>
+      <c r="C4" s="7" t="s">
+        <v>38</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>15</v>
@@ -723,7 +744,7 @@
       <c r="E4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>26</v>
       </c>
     </row>
@@ -734,8 +755,8 @@
       <c r="B5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="5">
-        <v>27406</v>
+      <c r="C5" s="7" t="s">
+        <v>39</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>20</v>
@@ -743,7 +764,7 @@
       <c r="E5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>30</v>
       </c>
     </row>
@@ -754,8 +775,8 @@
       <c r="B6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="5">
-        <v>40359</v>
+      <c r="C6" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>32</v>
@@ -763,11 +784,12 @@
       <c r="E6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="5" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="F6" r:id="rId1" display="mailto:kiran.kumar@gmail.com" xr:uid="{8E4FF1C4-A486-4E00-8CAC-5B0751AA02CA}"/>
     <hyperlink ref="F5" r:id="rId2" display="mailto:lakshmi.devi@gmail.com" xr:uid="{56886F69-2DA0-4471-BC73-857F2BD266E1}"/>

</xml_diff>

<commit_message>
feature/MyAccountMod: add final changes with all test cases passing
</commit_message>
<xml_diff>
--- a/src/test/resources/Reader/Apollo247_TestData.xlsx
+++ b/src/test/resources/Reader/Apollo247_TestData.xlsx
@@ -4,13 +4,15 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2448" windowWidth="8436" windowHeight="2448" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="BMI" sheetId="1" r:id="rId1"/>
-    <sheet name="FamilyMembers" sheetId="2" r:id="rId2"/>
+    <sheet name="Patients_Data" sheetId="2" r:id="rId2"/>
+    <sheet name="FamilyMembers" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:H7"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,12 +22,126 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Height</t>
-  </si>
-  <si>
-    <t>Weight</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="49">
+  <si>
+    <t>Height (ft)</t>
+  </si>
+  <si>
+    <t>Weight (kg)</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Underweight</t>
+  </si>
+  <si>
+    <t>Overweight</t>
+  </si>
+  <si>
+    <t>Obese</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>DateOfBirth</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Relation</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Brother</t>
+  </si>
+  <si>
+    <t>rahul.kumar@gmail.com</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>Sharma</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Sister</t>
+  </si>
+  <si>
+    <t>priya.sharma@gmail.com</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>Reddy</t>
+  </si>
+  <si>
+    <t>Father</t>
+  </si>
+  <si>
+    <t>arjun.reddy@gmail.com</t>
+  </si>
+  <si>
+    <t>Lakshmi</t>
+  </si>
+  <si>
+    <t>Devi</t>
+  </si>
+  <si>
+    <t>Mother</t>
+  </si>
+  <si>
+    <t>lakshmi.devi@gmail.com</t>
+  </si>
+  <si>
+    <t>Kiran</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Son</t>
+  </si>
+  <si>
+    <t>kiran.kumar@gmail.com</t>
+  </si>
+  <si>
+    <t>12/03/2002</t>
+  </si>
+  <si>
+    <t>12/03/2006</t>
+  </si>
+  <si>
+    <t>15/02/2000</t>
+  </si>
+  <si>
+    <t>12/11/1998</t>
+  </si>
+  <si>
+    <t>01/07/2008</t>
   </si>
   <si>
     <t>firstName</t>
@@ -37,29 +153,54 @@
     <t>dob</t>
   </si>
   <si>
+    <t>Vishva</t>
+  </si>
+  <si>
     <t>D</t>
   </si>
   <si>
+    <t>Prithvi</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
-    <t>Prithvi</t>
-  </si>
-  <si>
-    <t>Vishva</t>
-  </si>
-  <si>
-    <t>30-02-2000</t>
+    <t>31/05/1998</t>
+  </si>
+  <si>
+    <t>12/03/2004</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -73,7 +214,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -81,15 +222,55 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -368,42 +549,133 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>170</v>
-      </c>
-      <c r="B2">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>5.7</v>
+      </c>
+      <c r="B2" s="2">
+        <v>65</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2">
+        <v>50</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="B4" s="2">
+        <v>70</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>5.8</v>
+      </c>
+      <c r="B5" s="2">
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>160</v>
-      </c>
-      <c r="B3">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>155</v>
-      </c>
-      <c r="B4">
+      <c r="C5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5.2</v>
+      </c>
+      <c r="B6" s="2">
         <v>45</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6.1</v>
+      </c>
+      <c r="B7" s="2">
+        <v>90</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>5.9</v>
+      </c>
+      <c r="B9" s="2">
+        <v>75</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>5.7</v>
+      </c>
+      <c r="B10" s="2">
+        <v>101</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>6</v>
+      </c>
+      <c r="B11" s="2">
+        <v>106</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -413,43 +685,187 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="F6" r:id="rId1" display="mailto:kiran.kumar@gmail.com"/>
+    <hyperlink ref="F5" r:id="rId2" display="mailto:lakshmi.devi@gmail.com"/>
+    <hyperlink ref="F4" r:id="rId3" display="mailto:arjun.reddy@gmail.com"/>
+    <hyperlink ref="F3" r:id="rId4" display="mailto:priya.sharma@gmail.com"/>
+    <hyperlink ref="F2" r:id="rId5" display="mailto:rahul.kumar@gmail.com"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <v>37508</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(labtest) : fixed minute bugs and fixed explicit waits to handle dynamic webelements
</commit_message>
<xml_diff>
--- a/src/test/resources/Reader/Apollo247_TestData.xlsx
+++ b/src/test/resources/Reader/Apollo247_TestData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shyam Sundar\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE1200AA-3320-4C2B-BF0F-F0EE70AC6368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A18B651-A12A-4DE8-8625-DD72358DC96C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BMI" sheetId="1" r:id="rId1"/>
     <sheet name="Patients_Data" sheetId="2" r:id="rId2"/>
+    <sheet name="FamilyMembers" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="49">
   <si>
     <t>Height (ft)</t>
   </si>
@@ -146,6 +147,33 @@
   </si>
   <si>
     <t>01/07/2008</t>
+  </si>
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>Vishva</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Prithvi</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>31/05/1998</t>
+  </si>
+  <si>
+    <t>12/03/2004</t>
   </si>
 </sst>
 </file>
@@ -219,7 +247,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -242,6 +270,9 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -799,4 +830,50 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BE65286-7997-4135-A8D2-DDAC29E69C7A}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="10.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix : updated excel to fetch data for data drivern testing
</commit_message>
<xml_diff>
--- a/src/test/resources/Reader/Apollo247_TestData.xlsx
+++ b/src/test/resources/Reader/Apollo247_TestData.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shyam Sundar\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7813A325-64A3-4197-88EB-6113563BB9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1742AD06-6983-47BA-93C3-C31A762C4029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BMI" sheetId="1" r:id="rId1"/>
-    <sheet name="Patients_Data" sheetId="2" r:id="rId2"/>
-    <sheet name="FamilyMembers" sheetId="3" r:id="rId3"/>
-    <sheet name="Policy_purchase_Data" sheetId="4" r:id="rId4"/>
+    <sheet name="BuyMedicine" sheetId="5" r:id="rId2"/>
+    <sheet name="Patients_Data" sheetId="2" r:id="rId3"/>
+    <sheet name="FamilyMembers" sheetId="3" r:id="rId4"/>
+    <sheet name="Policy_purchase_Data" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="284">
   <si>
     <t>Height (ft)</t>
   </si>
@@ -859,6 +860,27 @@
   </si>
   <si>
     <t>ProposerFN</t>
+  </si>
+  <si>
+    <t>MEDICINE NAME</t>
+  </si>
+  <si>
+    <t>Calpol 650</t>
+  </si>
+  <si>
+    <t>Digene Tablet</t>
+  </si>
+  <si>
+    <t>Gelusil Syrup</t>
+  </si>
+  <si>
+    <t>Benadryl Syrup</t>
+  </si>
+  <si>
+    <t>Vicks VapoRub</t>
+  </si>
+  <si>
+    <t>Moov Spray</t>
   </si>
 </sst>
 </file>
@@ -1182,19 +1204,28 @@
     <xf numFmtId="49" fontId="7" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1205,15 +1236,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1638,6 +1660,54 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B46A366B-4A49-4F81-9245-154B6D9B7EE7}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FECFBD-25D6-4F6C-91BB-5A6C18ADD79D}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:F6"/>
@@ -1782,7 +1852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BE65286-7997-4135-A8D2-DDAC29E69C7A}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C3"/>
@@ -1829,7 +1899,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F6F6BB4-2A7A-4EE8-A91D-627425662417}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A2:AU12"/>
@@ -1879,7 +1949,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="40" t="s">
         <v>49</v>
       </c>
       <c r="B2" s="41"/>
@@ -1930,7 +2000,7 @@
       <c r="AU2" s="41"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="42" t="s">
         <v>50</v>
       </c>
       <c r="B3" s="41"/>
@@ -1940,7 +2010,7 @@
       </c>
       <c r="E3" s="41"/>
       <c r="F3" s="41"/>
-      <c r="G3" s="46" t="s">
+      <c r="G3" s="49" t="s">
         <v>52</v>
       </c>
       <c r="H3" s="41"/>
@@ -1948,36 +2018,36 @@
       <c r="J3" s="41"/>
       <c r="K3" s="41"/>
       <c r="L3" s="41"/>
-      <c r="M3" s="47" t="s">
+      <c r="M3" s="50" t="s">
         <v>53</v>
       </c>
       <c r="N3" s="41"/>
       <c r="O3" s="41"/>
       <c r="P3" s="41"/>
       <c r="Q3" s="41"/>
-      <c r="R3" s="43" t="s">
+      <c r="R3" s="47" t="s">
         <v>54</v>
       </c>
       <c r="S3" s="41"/>
       <c r="T3" s="41"/>
       <c r="U3" s="41"/>
       <c r="V3" s="41"/>
-      <c r="W3" s="51" t="s">
+      <c r="W3" s="43" t="s">
         <v>55</v>
       </c>
       <c r="X3" s="41"/>
       <c r="Y3" s="41"/>
-      <c r="Z3" s="45" t="s">
+      <c r="Z3" s="48" t="s">
         <v>56</v>
       </c>
       <c r="AA3" s="41"/>
       <c r="AB3" s="41"/>
-      <c r="AC3" s="48" t="s">
+      <c r="AC3" s="51" t="s">
         <v>57</v>
       </c>
       <c r="AD3" s="41"/>
       <c r="AE3" s="41"/>
-      <c r="AF3" s="42" t="s">
+      <c r="AF3" s="46" t="s">
         <v>58</v>
       </c>
       <c r="AG3" s="41"/>
@@ -1987,7 +2057,7 @@
       <c r="AK3" s="41"/>
       <c r="AL3" s="41"/>
       <c r="AM3" s="41"/>
-      <c r="AN3" s="50" t="s">
+      <c r="AN3" s="42" t="s">
         <v>59</v>
       </c>
       <c r="AO3" s="41"/>
@@ -2835,7 +2905,7 @@
       </c>
     </row>
     <row r="11" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="45" t="s">
         <v>218</v>
       </c>
       <c r="B11" s="41"/>
@@ -3030,11 +3100,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A2:AU2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="AN3:AP3"/>
-    <mergeCell ref="AQ3:AU3"/>
     <mergeCell ref="A11:AU11"/>
     <mergeCell ref="AF3:AM3"/>
     <mergeCell ref="R3:V3"/>
@@ -3043,6 +3108,11 @@
     <mergeCell ref="G3:L3"/>
     <mergeCell ref="M3:Q3"/>
     <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="A2:AU2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="AN3:AP3"/>
+    <mergeCell ref="AQ3:AU3"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix : fixed bugs and minor syntax
</commit_message>
<xml_diff>
--- a/src/test/resources/Reader/Apollo247_TestData.xlsx
+++ b/src/test/resources/Reader/Apollo247_TestData.xlsx
@@ -3,14 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shyam Sundar\OneDrive\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1742AD06-6983-47BA-93C3-C31A762C4029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C2314B8E-F19B-46CE-AD1F-0D6C2D0F43D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BMI" sheetId="1" r:id="rId1"/>
@@ -19,7 +14,8 @@
     <sheet name="FamilyMembers" sheetId="3" r:id="rId4"/>
     <sheet name="Policy_purchase_Data" sheetId="4" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:L19"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1204,38 +1200,38 @@
     <xf numFmtId="49" fontId="7" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1949,7 +1945,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="49" t="s">
         <v>49</v>
       </c>
       <c r="B2" s="41"/>
@@ -2000,7 +1996,7 @@
       <c r="AU2" s="41"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="50" t="s">
         <v>50</v>
       </c>
       <c r="B3" s="41"/>
@@ -2010,7 +2006,7 @@
       </c>
       <c r="E3" s="41"/>
       <c r="F3" s="41"/>
-      <c r="G3" s="49" t="s">
+      <c r="G3" s="46" t="s">
         <v>52</v>
       </c>
       <c r="H3" s="41"/>
@@ -2018,36 +2014,36 @@
       <c r="J3" s="41"/>
       <c r="K3" s="41"/>
       <c r="L3" s="41"/>
-      <c r="M3" s="50" t="s">
+      <c r="M3" s="47" t="s">
         <v>53</v>
       </c>
       <c r="N3" s="41"/>
       <c r="O3" s="41"/>
       <c r="P3" s="41"/>
       <c r="Q3" s="41"/>
-      <c r="R3" s="47" t="s">
+      <c r="R3" s="43" t="s">
         <v>54</v>
       </c>
       <c r="S3" s="41"/>
       <c r="T3" s="41"/>
       <c r="U3" s="41"/>
       <c r="V3" s="41"/>
-      <c r="W3" s="43" t="s">
+      <c r="W3" s="51" t="s">
         <v>55</v>
       </c>
       <c r="X3" s="41"/>
       <c r="Y3" s="41"/>
-      <c r="Z3" s="48" t="s">
+      <c r="Z3" s="45" t="s">
         <v>56</v>
       </c>
       <c r="AA3" s="41"/>
       <c r="AB3" s="41"/>
-      <c r="AC3" s="51" t="s">
+      <c r="AC3" s="48" t="s">
         <v>57</v>
       </c>
       <c r="AD3" s="41"/>
       <c r="AE3" s="41"/>
-      <c r="AF3" s="46" t="s">
+      <c r="AF3" s="42" t="s">
         <v>58</v>
       </c>
       <c r="AG3" s="41"/>
@@ -2057,7 +2053,7 @@
       <c r="AK3" s="41"/>
       <c r="AL3" s="41"/>
       <c r="AM3" s="41"/>
-      <c r="AN3" s="42" t="s">
+      <c r="AN3" s="50" t="s">
         <v>59</v>
       </c>
       <c r="AO3" s="41"/>
@@ -2905,7 +2901,7 @@
       </c>
     </row>
     <row r="11" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A11" s="45" t="s">
+      <c r="A11" s="40" t="s">
         <v>218</v>
       </c>
       <c r="B11" s="41"/>
@@ -3100,6 +3096,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A2:AU2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="AN3:AP3"/>
+    <mergeCell ref="AQ3:AU3"/>
     <mergeCell ref="A11:AU11"/>
     <mergeCell ref="AF3:AM3"/>
     <mergeCell ref="R3:V3"/>
@@ -3108,11 +3109,6 @@
     <mergeCell ref="G3:L3"/>
     <mergeCell ref="M3:Q3"/>
     <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="A2:AU2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="AN3:AP3"/>
-    <mergeCell ref="AQ3:AU3"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>